<commit_message>
update general sin cuadernos de queseria
por necesidad de reorganizar contenido
</commit_message>
<xml_diff>
--- a/datos/2025-11-06-ejemplo-std-tecnico.xlsx
+++ b/datos/2025-11-06-ejemplo-std-tecnico.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29721"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/34bf2af71bbc2e43/Documentos/GitHub/master-queseria/website/datos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="958" documentId="8_{5F9E455A-213A-447C-A11C-7E9616724FEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{89322A96-2EFD-4D10-80FE-1DDAA778226C}"/>
+  <xr:revisionPtr revIDLastSave="959" documentId="8_{5F9E455A-213A-447C-A11C-7E9616724FEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1D9DDED1-E90C-4CC9-8D4B-8C486BDEE985}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="675" xr2:uid="{6977E7F1-D64B-47FE-B2A7-D4E9B0399E18}"/>
   </bookViews>
@@ -712,7 +712,7 @@
     <definedName name="zzzzzzzzzzzzzzzzzz" localSheetId="0" hidden="1">{"QQQ",#N/A,FALSE,"RIEP"}</definedName>
     <definedName name="zzzzzzzzzzzzzzzzzz" hidden="1">{"QQQ",#N/A,FALSE,"RIEP"}</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -724,6 +724,8 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -733,134 +735,134 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
   <si>
+    <t>Estándar de producto</t>
+  </si>
+  <si>
+    <t>Fórmulas</t>
+  </si>
+  <si>
+    <t>Vaca</t>
+  </si>
+  <si>
+    <t>Mezcla</t>
+  </si>
+  <si>
+    <t>Oveja</t>
+  </si>
+  <si>
+    <t>Bajo en MG</t>
+  </si>
+  <si>
+    <t>Mozza</t>
+  </si>
+  <si>
+    <t>Fabricación, KG</t>
+  </si>
+  <si>
+    <t>1. Características del queso</t>
+  </si>
+  <si>
+    <t>EST salida salado</t>
+  </si>
+  <si>
+    <t>MG salida salado</t>
+  </si>
+  <si>
     <t>ESM</t>
   </si>
   <si>
+    <t>=B4-B5</t>
+  </si>
+  <si>
+    <t>HFD</t>
+  </si>
+  <si>
+    <t>=(1-B4)/(1-B5)</t>
+  </si>
+  <si>
+    <t>G/ES</t>
+  </si>
+  <si>
+    <t>=B5/B4</t>
+  </si>
+  <si>
+    <t>2. Composición de la leche de fabricación</t>
+  </si>
+  <si>
+    <t>Leche en cuba MG (g/L)</t>
+  </si>
+  <si>
+    <t>Leche en cuba MP (g/L)</t>
+  </si>
+  <si>
+    <t>3. Datos tecnológicos</t>
+  </si>
+  <si>
+    <t>Recup MP (dato real de la fabricación)</t>
+  </si>
+  <si>
+    <t>4. Cálculos</t>
+  </si>
+  <si>
+    <t>ESM queso obtenido a partir de MP leche (g/L)</t>
+  </si>
+  <si>
+    <t>=B13*B11</t>
+  </si>
+  <si>
     <t>Litraje unitario</t>
   </si>
   <si>
+    <t>=B6*1000/B15</t>
+  </si>
+  <si>
     <t>MG teórica en la cuba (g/L)</t>
   </si>
   <si>
-    <t>Mezcla</t>
-  </si>
-  <si>
-    <t>Vaca</t>
-  </si>
-  <si>
-    <t>Oveja</t>
-  </si>
-  <si>
-    <t>Bajo en MG</t>
-  </si>
-  <si>
-    <t>Fabricación, KG</t>
-  </si>
-  <si>
-    <t>HFD</t>
-  </si>
-  <si>
-    <t>G/ES</t>
+    <t>=B5*1000/B16</t>
   </si>
   <si>
     <t>Recup MG</t>
   </si>
   <si>
+    <t>=B17/B10</t>
+  </si>
+  <si>
+    <t>MG pérdida bruta en suero (g/L)</t>
+  </si>
+  <si>
+    <t>=B17-B10</t>
+  </si>
+  <si>
+    <t>MG pérdida bruta en suero %</t>
+  </si>
+  <si>
+    <t>=B19/B10</t>
+  </si>
+  <si>
+    <t>Consumo MG/kg queso</t>
+  </si>
+  <si>
+    <t>=B10*B16</t>
+  </si>
+  <si>
     <t>Consumo MP/kg queso</t>
   </si>
   <si>
-    <t>MG pérdida bruta en suero %</t>
-  </si>
-  <si>
-    <t>Consumo MG/kg queso</t>
-  </si>
-  <si>
-    <t>Estándar de producto</t>
-  </si>
-  <si>
-    <t>ESM queso obtenido a partir de MP leche (g/L)</t>
-  </si>
-  <si>
-    <t>MG pérdida bruta en suero (g/L)</t>
-  </si>
-  <si>
-    <t>Leche en cuba MG (g/L)</t>
-  </si>
-  <si>
-    <t>Leche en cuba MP (g/L)</t>
-  </si>
-  <si>
-    <t>=B4-B5</t>
-  </si>
-  <si>
-    <t>=(1-B4)/(1-B5)</t>
-  </si>
-  <si>
-    <t>=B5/B4</t>
-  </si>
-  <si>
-    <t>Fórmulas</t>
-  </si>
-  <si>
-    <t>=B13*B11</t>
-  </si>
-  <si>
-    <t>=B6*1000/B15</t>
-  </si>
-  <si>
-    <t>=B5*1000/B16</t>
-  </si>
-  <si>
-    <t>=B17/B10</t>
-  </si>
-  <si>
-    <t>=B17-B10</t>
-  </si>
-  <si>
-    <t>=B19/B10</t>
-  </si>
-  <si>
-    <t>=B10*B16</t>
-  </si>
-  <si>
     <t>=B11*B16</t>
-  </si>
-  <si>
-    <t>Recup MP (dato real de la fabricación)</t>
-  </si>
-  <si>
-    <t>EST salida salado</t>
-  </si>
-  <si>
-    <t>MG salida salado</t>
-  </si>
-  <si>
-    <t>1. Características del queso</t>
-  </si>
-  <si>
-    <t>2. Composición de la leche de fabricación</t>
-  </si>
-  <si>
-    <t>3. Datos tecnológicos</t>
-  </si>
-  <si>
-    <t>4. Cálculos</t>
-  </si>
-  <si>
-    <t>Mozza</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <numFmts count="4">
     <numFmt numFmtId="164" formatCode="#,##0_ ;[Red]\-#,##0\ "/>
     <numFmt numFmtId="165" formatCode="#,##0.000_ ;[Red]\-#,##0.000\ "/>
     <numFmt numFmtId="166" formatCode="_-* #,##0.00\ _€_-;\-* #,##0.00\ _€_-;_-* &quot;-&quot;??\ _€_-;_-@_-"/>
     <numFmt numFmtId="167" formatCode="#,##0.00_ ;[Red]\-#,##0.00\ "/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1088,7 +1090,9 @@
     <cellStyle name="Porcentaje" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
+    <tableStyle name="Invisible" pivot="0" table="0" count="0" xr9:uid="{28C21CB3-7664-42D2-9D67-4CB284AD2D41}"/>
+  </tableStyles>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1129,13 +1133,7 @@
     </sheetNames>
     <sheetDataSet>
       <sheetData sheetId="0" refreshError="1"/>
-      <sheetData sheetId="1">
-        <row r="10">
-          <cell r="B10" t="str">
-            <v>2010</v>
-          </cell>
-        </row>
-      </sheetData>
+      <sheetData sheetId="1"/>
       <sheetData sheetId="2" refreshError="1"/>
       <sheetData sheetId="3" refreshError="1"/>
       <sheetData sheetId="4" refreshError="1"/>
@@ -1145,53 +1143,17 @@
       <sheetData sheetId="8" refreshError="1"/>
       <sheetData sheetId="9" refreshError="1"/>
       <sheetData sheetId="10" refreshError="1"/>
-      <sheetData sheetId="11">
-        <row r="6">
-          <cell r="O6">
-            <v>29.297000000000001</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="12">
-        <row r="73">
-          <cell r="G73">
-            <v>1.54</v>
-          </cell>
-        </row>
-      </sheetData>
+      <sheetData sheetId="11"/>
+      <sheetData sheetId="12"/>
       <sheetData sheetId="13" refreshError="1"/>
-      <sheetData sheetId="14">
-        <row r="258">
-          <cell r="F258">
-            <v>2.2000000000000002</v>
-          </cell>
-        </row>
-      </sheetData>
+      <sheetData sheetId="14"/>
       <sheetData sheetId="15"/>
-      <sheetData sheetId="16">
-        <row r="270">
-          <cell r="C270" t="str">
-            <v>E1</v>
-          </cell>
-        </row>
-      </sheetData>
+      <sheetData sheetId="16"/>
       <sheetData sheetId="17" refreshError="1"/>
       <sheetData sheetId="18" refreshError="1"/>
-      <sheetData sheetId="19">
-        <row r="9">
-          <cell r="AD9">
-            <v>4.3841000000000001</v>
-          </cell>
-        </row>
-      </sheetData>
+      <sheetData sheetId="19"/>
       <sheetData sheetId="20" refreshError="1"/>
-      <sheetData sheetId="21">
-        <row r="3">
-          <cell r="E3" t="str">
-            <v>JAN2010</v>
-          </cell>
-        </row>
-      </sheetData>
+      <sheetData sheetId="21"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -1248,444 +1210,15 @@
       <sheetData sheetId="6"/>
       <sheetData sheetId="7"/>
       <sheetData sheetId="8"/>
-      <sheetData sheetId="9" refreshError="1">
-        <row r="2">
-          <cell r="A2" t="str">
-            <v>January 2008</v>
-          </cell>
-        </row>
-        <row r="3">
-          <cell r="A3" t="str">
-            <v>February 2008</v>
-          </cell>
-        </row>
-        <row r="4">
-          <cell r="A4" t="str">
-            <v>March 2008</v>
-          </cell>
-        </row>
-        <row r="5">
-          <cell r="A5" t="str">
-            <v>April 2008</v>
-          </cell>
-        </row>
-        <row r="6">
-          <cell r="A6" t="str">
-            <v>May 2008</v>
-          </cell>
-        </row>
-        <row r="7">
-          <cell r="A7" t="str">
-            <v>June 2008</v>
-          </cell>
-        </row>
-        <row r="8">
-          <cell r="A8" t="str">
-            <v>July 2008</v>
-          </cell>
-        </row>
-        <row r="9">
-          <cell r="A9" t="str">
-            <v>August 2008</v>
-          </cell>
-        </row>
-        <row r="10">
-          <cell r="A10" t="str">
-            <v>September 2008</v>
-          </cell>
-        </row>
-        <row r="11">
-          <cell r="A11" t="str">
-            <v>October 2008</v>
-          </cell>
-        </row>
-        <row r="12">
-          <cell r="A12" t="str">
-            <v>November 2008</v>
-          </cell>
-        </row>
-        <row r="13">
-          <cell r="A13" t="str">
-            <v>December 2008</v>
-          </cell>
-        </row>
-        <row r="14">
-          <cell r="A14" t="str">
-            <v>January 2009</v>
-          </cell>
-        </row>
-        <row r="15">
-          <cell r="A15" t="str">
-            <v>February 2009</v>
-          </cell>
-        </row>
-        <row r="16">
-          <cell r="A16" t="str">
-            <v>March 2009</v>
-          </cell>
-        </row>
-        <row r="17">
-          <cell r="A17" t="str">
-            <v>April 2009</v>
-          </cell>
-        </row>
-        <row r="18">
-          <cell r="A18" t="str">
-            <v>May 2009</v>
-          </cell>
-        </row>
-        <row r="19">
-          <cell r="A19" t="str">
-            <v>June 2009</v>
-          </cell>
-        </row>
-        <row r="20">
-          <cell r="A20" t="str">
-            <v>July 2009</v>
-          </cell>
-        </row>
-        <row r="21">
-          <cell r="A21" t="str">
-            <v>August 2009</v>
-          </cell>
-        </row>
-        <row r="22">
-          <cell r="A22" t="str">
-            <v>September 2009</v>
-          </cell>
-        </row>
-        <row r="23">
-          <cell r="A23" t="str">
-            <v>October 2009</v>
-          </cell>
-        </row>
-        <row r="24">
-          <cell r="A24" t="str">
-            <v>November 2009</v>
-          </cell>
-        </row>
-        <row r="25">
-          <cell r="A25" t="str">
-            <v>December 2009</v>
-          </cell>
-        </row>
-      </sheetData>
+      <sheetData sheetId="9" refreshError="1"/>
       <sheetData sheetId="10"/>
-      <sheetData sheetId="11" refreshError="1">
-        <row r="2">
-          <cell r="A2" t="str">
-            <v>January 2008</v>
-          </cell>
-        </row>
-        <row r="3">
-          <cell r="A3" t="str">
-            <v>February 2008</v>
-          </cell>
-        </row>
-        <row r="4">
-          <cell r="A4" t="str">
-            <v>March 2008</v>
-          </cell>
-        </row>
-        <row r="5">
-          <cell r="A5" t="str">
-            <v>April 2008</v>
-          </cell>
-        </row>
-        <row r="6">
-          <cell r="A6" t="str">
-            <v>May 2008</v>
-          </cell>
-        </row>
-        <row r="7">
-          <cell r="A7" t="str">
-            <v>June 2008</v>
-          </cell>
-        </row>
-        <row r="8">
-          <cell r="A8" t="str">
-            <v>July 2008</v>
-          </cell>
-        </row>
-        <row r="9">
-          <cell r="A9" t="str">
-            <v>August 2008</v>
-          </cell>
-        </row>
-        <row r="10">
-          <cell r="A10" t="str">
-            <v>September 2008</v>
-          </cell>
-        </row>
-        <row r="11">
-          <cell r="A11" t="str">
-            <v>October 2008</v>
-          </cell>
-        </row>
-        <row r="12">
-          <cell r="A12" t="str">
-            <v>November 2008</v>
-          </cell>
-        </row>
-        <row r="13">
-          <cell r="A13" t="str">
-            <v>December 2008</v>
-          </cell>
-        </row>
-        <row r="14">
-          <cell r="A14" t="str">
-            <v>January 2009</v>
-          </cell>
-        </row>
-        <row r="15">
-          <cell r="A15" t="str">
-            <v>February 2009</v>
-          </cell>
-        </row>
-        <row r="16">
-          <cell r="A16" t="str">
-            <v>March 2009</v>
-          </cell>
-        </row>
-        <row r="17">
-          <cell r="A17" t="str">
-            <v>April 2009</v>
-          </cell>
-        </row>
-        <row r="18">
-          <cell r="A18" t="str">
-            <v>May 2009</v>
-          </cell>
-        </row>
-        <row r="19">
-          <cell r="A19" t="str">
-            <v>June 2009</v>
-          </cell>
-        </row>
-        <row r="20">
-          <cell r="A20" t="str">
-            <v>July 2009</v>
-          </cell>
-        </row>
-        <row r="21">
-          <cell r="A21" t="str">
-            <v>August 2009</v>
-          </cell>
-        </row>
-        <row r="22">
-          <cell r="A22" t="str">
-            <v>September 2009</v>
-          </cell>
-        </row>
-        <row r="23">
-          <cell r="A23" t="str">
-            <v>October 2009</v>
-          </cell>
-        </row>
-        <row r="24">
-          <cell r="A24" t="str">
-            <v>November 2009</v>
-          </cell>
-        </row>
-        <row r="25">
-          <cell r="A25" t="str">
-            <v>December 2009</v>
-          </cell>
-        </row>
-      </sheetData>
+      <sheetData sheetId="11" refreshError="1"/>
       <sheetData sheetId="12"/>
-      <sheetData sheetId="13" refreshError="1">
-        <row r="2">
-          <cell r="A2" t="str">
-            <v>January 2008</v>
-          </cell>
-        </row>
-        <row r="3">
-          <cell r="A3" t="str">
-            <v>February 2008</v>
-          </cell>
-        </row>
-        <row r="4">
-          <cell r="A4" t="str">
-            <v>March 2008</v>
-          </cell>
-        </row>
-        <row r="5">
-          <cell r="A5" t="str">
-            <v>April 2008</v>
-          </cell>
-        </row>
-        <row r="6">
-          <cell r="A6" t="str">
-            <v>May 2008</v>
-          </cell>
-        </row>
-        <row r="7">
-          <cell r="A7" t="str">
-            <v>June 2008</v>
-          </cell>
-        </row>
-        <row r="8">
-          <cell r="A8" t="str">
-            <v>July 2008</v>
-          </cell>
-        </row>
-        <row r="9">
-          <cell r="A9" t="str">
-            <v>August 2008</v>
-          </cell>
-        </row>
-        <row r="10">
-          <cell r="A10" t="str">
-            <v>September 2008</v>
-          </cell>
-        </row>
-        <row r="11">
-          <cell r="A11" t="str">
-            <v>October 2008</v>
-          </cell>
-        </row>
-        <row r="12">
-          <cell r="A12" t="str">
-            <v>November 2008</v>
-          </cell>
-        </row>
-        <row r="13">
-          <cell r="A13" t="str">
-            <v>December 2008</v>
-          </cell>
-        </row>
-        <row r="14">
-          <cell r="A14" t="str">
-            <v>January 2009</v>
-          </cell>
-        </row>
-        <row r="15">
-          <cell r="A15" t="str">
-            <v>February 2009</v>
-          </cell>
-        </row>
-        <row r="16">
-          <cell r="A16" t="str">
-            <v>March 2009</v>
-          </cell>
-        </row>
-        <row r="17">
-          <cell r="A17" t="str">
-            <v>April 2009</v>
-          </cell>
-        </row>
-        <row r="18">
-          <cell r="A18" t="str">
-            <v>May 2009</v>
-          </cell>
-        </row>
-        <row r="19">
-          <cell r="A19" t="str">
-            <v>June 2009</v>
-          </cell>
-        </row>
-        <row r="20">
-          <cell r="A20" t="str">
-            <v>July 2009</v>
-          </cell>
-        </row>
-        <row r="21">
-          <cell r="A21" t="str">
-            <v>August 2009</v>
-          </cell>
-        </row>
-        <row r="22">
-          <cell r="A22" t="str">
-            <v>September 2009</v>
-          </cell>
-        </row>
-        <row r="23">
-          <cell r="A23" t="str">
-            <v>October 2009</v>
-          </cell>
-        </row>
-        <row r="24">
-          <cell r="A24" t="str">
-            <v>November 2009</v>
-          </cell>
-        </row>
-        <row r="25">
-          <cell r="A25" t="str">
-            <v>December 2009</v>
-          </cell>
-        </row>
-      </sheetData>
+      <sheetData sheetId="13" refreshError="1"/>
       <sheetData sheetId="14"/>
       <sheetData sheetId="15"/>
       <sheetData sheetId="16"/>
-      <sheetData sheetId="17" refreshError="1">
-        <row r="2">
-          <cell r="A2" t="str">
-            <v>December 2008</v>
-          </cell>
-        </row>
-        <row r="3">
-          <cell r="A3" t="str">
-            <v>January 2009</v>
-          </cell>
-        </row>
-        <row r="4">
-          <cell r="A4" t="str">
-            <v>February 2009</v>
-          </cell>
-        </row>
-        <row r="5">
-          <cell r="A5" t="str">
-            <v>March 2009</v>
-          </cell>
-        </row>
-        <row r="6">
-          <cell r="A6" t="str">
-            <v>April 2009</v>
-          </cell>
-        </row>
-        <row r="7">
-          <cell r="A7" t="str">
-            <v>May 2009</v>
-          </cell>
-        </row>
-        <row r="8">
-          <cell r="A8" t="str">
-            <v>June 2009</v>
-          </cell>
-        </row>
-        <row r="9">
-          <cell r="A9" t="str">
-            <v>July 2009</v>
-          </cell>
-        </row>
-        <row r="10">
-          <cell r="A10" t="str">
-            <v>August 2009</v>
-          </cell>
-        </row>
-        <row r="11">
-          <cell r="A11" t="str">
-            <v>September 2009</v>
-          </cell>
-        </row>
-        <row r="12">
-          <cell r="A12" t="str">
-            <v>October 2009</v>
-          </cell>
-        </row>
-        <row r="13">
-          <cell r="A13" t="str">
-            <v>November 2009</v>
-          </cell>
-        </row>
-        <row r="14">
-          <cell r="A14" t="str">
-            <v>December 2009</v>
-          </cell>
-        </row>
-      </sheetData>
+      <sheetData sheetId="17" refreshError="1"/>
       <sheetData sheetId="18"/>
       <sheetData sheetId="19"/>
       <sheetData sheetId="20"/>
@@ -1728,13 +1261,7 @@
     </sheetNames>
     <sheetDataSet>
       <sheetData sheetId="0"/>
-      <sheetData sheetId="1" refreshError="1">
-        <row r="4">
-          <cell r="A4" t="str">
-            <v>__Amount_for_Monthly_1</v>
-          </cell>
-        </row>
-      </sheetData>
+      <sheetData sheetId="1" refreshError="1"/>
       <sheetData sheetId="2"/>
       <sheetData sheetId="3"/>
       <sheetData sheetId="4"/>
@@ -1818,917 +1345,7 @@
       <sheetName val="DATA"/>
     </sheetNames>
     <sheetDataSet>
-      <sheetData sheetId="0" refreshError="1">
-        <row r="2">
-          <cell r="B2" t="str">
-            <v xml:space="preserve"> Stabilimento di</v>
-          </cell>
-          <cell r="H2" t="str">
-            <v>SCHEDA RILEVAZIONE TEMPI</v>
-          </cell>
-          <cell r="O2" t="str">
-            <v xml:space="preserve"> Data :</v>
-          </cell>
-        </row>
-        <row r="3">
-          <cell r="B3" t="str">
-            <v xml:space="preserve"> CERTOSA </v>
-          </cell>
-          <cell r="D3">
-            <v>220</v>
-          </cell>
-          <cell r="F3" t="str">
-            <v>Reparto :</v>
-          </cell>
-          <cell r="G3" t="str">
-            <v>FUSI</v>
-          </cell>
-          <cell r="H3">
-            <v>210</v>
-          </cell>
-          <cell r="I3" t="str">
-            <v>PREPARAZIONE IMPASTI E FUSIONE</v>
-          </cell>
-          <cell r="O3" t="str">
-            <v xml:space="preserve"> Gennaio 2004</v>
-          </cell>
-        </row>
-        <row r="4">
-          <cell r="B4" t="str">
-            <v xml:space="preserve"> PRODUZIONE :</v>
-          </cell>
-          <cell r="D4" t="str">
-            <v xml:space="preserve">CREMA BEL PAESE  NORMALE + BIANCO + CREMOZOLA </v>
-          </cell>
-        </row>
-        <row r="5">
-          <cell r="D5" t="str">
-            <v>+ FILANTE + FILANTE x PIZZA + IDEA PIZZA + FORMAGGIO PER PIZZA</v>
-          </cell>
-        </row>
-        <row r="6">
-          <cell r="F6" t="str">
-            <v>Persone</v>
-          </cell>
-          <cell r="G6" t="str">
-            <v>Tempo impiegato</v>
-          </cell>
-          <cell r="J6" t="str">
-            <v>Quantità</v>
-          </cell>
-          <cell r="L6" t="str">
-            <v>Tempo</v>
-          </cell>
-          <cell r="M6" t="str">
-            <v>Prodotti destinatari</v>
-          </cell>
-        </row>
-        <row r="7">
-          <cell r="D7" t="str">
-            <v>OPERAZIONI</v>
-          </cell>
-          <cell r="F7" t="str">
-            <v>occupate</v>
-          </cell>
-          <cell r="G7" t="str">
-            <v>Ore</v>
-          </cell>
-          <cell r="H7" t="str">
-            <v>Ore</v>
-          </cell>
-          <cell r="I7" t="str">
-            <v>Totale</v>
-          </cell>
-          <cell r="L7" t="str">
-            <v>in ore</v>
-          </cell>
-          <cell r="M7" t="str">
-            <v>C.B.P.</v>
-          </cell>
-          <cell r="N7" t="str">
-            <v>C.B.P +.</v>
-          </cell>
-          <cell r="P7" t="str">
-            <v>Filante</v>
-          </cell>
-        </row>
-        <row r="8">
-          <cell r="F8" t="str">
-            <v>Posizioni</v>
-          </cell>
-          <cell r="G8" t="str">
-            <v>squadra</v>
-          </cell>
-          <cell r="H8" t="str">
-            <v>squadra</v>
-          </cell>
-          <cell r="I8" t="str">
-            <v>ore ind</v>
-          </cell>
-          <cell r="J8" t="str">
-            <v>Kg</v>
-          </cell>
-          <cell r="K8" t="str">
-            <v>Kg</v>
-          </cell>
-          <cell r="L8" t="str">
-            <v>riferito a</v>
-          </cell>
-          <cell r="M8" t="str">
-            <v>Normale</v>
-          </cell>
-          <cell r="N8" t="str">
-            <v>Dolc. Crem.</v>
-          </cell>
-          <cell r="O8" t="str">
-            <v>K 1</v>
-          </cell>
-          <cell r="P8" t="str">
-            <v>Idea Pizza</v>
-          </cell>
-        </row>
-        <row r="9">
-          <cell r="F9" t="str">
-            <v>occupate</v>
-          </cell>
-          <cell r="G9" t="str">
-            <v>in '</v>
-          </cell>
-          <cell r="H9" t="str">
-            <v>decimali</v>
-          </cell>
-          <cell r="I9" t="str">
-            <v>decimali</v>
-          </cell>
-          <cell r="J9" t="str">
-            <v>settimana</v>
-          </cell>
-          <cell r="K9" t="str">
-            <v>giorno</v>
-          </cell>
-          <cell r="L9" t="str">
-            <v>100 Kg</v>
-          </cell>
-          <cell r="N9" t="str">
-            <v xml:space="preserve">4 F-Proc.-Tir. </v>
-          </cell>
-          <cell r="P9" t="str">
-            <v>Rapè - Mozz.</v>
-          </cell>
-        </row>
-        <row r="11">
-          <cell r="G11" t="str">
-            <v xml:space="preserve"> x C.B.P. Normale</v>
-          </cell>
-          <cell r="J11" t="str">
-            <v xml:space="preserve"> x C.B.P. +  e  Dolcelatte Cremoso</v>
-          </cell>
-          <cell r="M11" t="str">
-            <v xml:space="preserve">  x Filante + Idea Pizza + Filante Rapè</v>
-          </cell>
-        </row>
-        <row r="12">
-          <cell r="C12" t="str">
-            <v xml:space="preserve"> Determinazione gg./anno lavorati</v>
-          </cell>
-          <cell r="G12" t="str">
-            <v>gg/sett.</v>
-          </cell>
-          <cell r="H12" t="str">
-            <v>sett/anno</v>
-          </cell>
-          <cell r="I12" t="str">
-            <v>gg/anno</v>
-          </cell>
-          <cell r="J12" t="str">
-            <v>gg/sett.</v>
-          </cell>
-          <cell r="K12" t="str">
-            <v>sett/anno</v>
-          </cell>
-          <cell r="L12" t="str">
-            <v>gg/anno</v>
-          </cell>
-          <cell r="M12" t="str">
-            <v>gg/sett.</v>
-          </cell>
-          <cell r="N12" t="str">
-            <v>sett/anno</v>
-          </cell>
-          <cell r="O12" t="str">
-            <v>gg/anno</v>
-          </cell>
-        </row>
-        <row r="15">
-          <cell r="G15">
-            <v>5</v>
-          </cell>
-          <cell r="H15">
-            <v>50</v>
-          </cell>
-          <cell r="I15">
-            <v>250</v>
-          </cell>
-          <cell r="J15">
-            <v>5</v>
-          </cell>
-          <cell r="K15">
-            <v>50</v>
-          </cell>
-          <cell r="L15">
-            <v>250</v>
-          </cell>
-          <cell r="M15">
-            <v>5</v>
-          </cell>
-          <cell r="N15">
-            <v>50</v>
-          </cell>
-          <cell r="O15">
-            <v>250</v>
-          </cell>
-        </row>
-        <row r="16">
-          <cell r="B16" t="str">
-            <v>A</v>
-          </cell>
-          <cell r="C16" t="str">
-            <v xml:space="preserve"> OPERAZIONI PRELIMINARI</v>
-          </cell>
-        </row>
-        <row r="17">
-          <cell r="M17" t="str">
-            <v xml:space="preserve">Tempo in ore riferito a 100/kg </v>
-          </cell>
-        </row>
-        <row r="18">
-          <cell r="B18">
-            <v>1</v>
-          </cell>
-          <cell r="C18" t="str">
-            <v xml:space="preserve"> Rifornimento materie prime a reparto :</v>
-          </cell>
-        </row>
-        <row r="19">
-          <cell r="C19" t="str">
-            <v xml:space="preserve"> - Scarico camions, pesatura palbox e stoccaggio in cella</v>
-          </cell>
-        </row>
-        <row r="20">
-          <cell r="C20" t="str">
-            <v xml:space="preserve"> - Prelievo campioni x analisi, controllo</v>
-          </cell>
-        </row>
-        <row r="21">
-          <cell r="C21" t="str">
-            <v xml:space="preserve">   rimanenze celle dinamica e formaggi</v>
-          </cell>
-          <cell r="F21">
-            <v>2</v>
-          </cell>
-          <cell r="G21">
-            <v>8</v>
-          </cell>
-          <cell r="H21">
-            <v>16</v>
-          </cell>
-          <cell r="I21">
-            <v>16</v>
-          </cell>
-          <cell r="K21">
-            <v>59868</v>
-          </cell>
-          <cell r="L21">
-            <v>2.6725462684572727E-2</v>
-          </cell>
-          <cell r="M21">
-            <v>2.6725462684572727E-2</v>
-          </cell>
-          <cell r="N21">
-            <v>2.6725462684572727E-2</v>
-          </cell>
-          <cell r="O21">
-            <v>2.6725462684572727E-2</v>
-          </cell>
-          <cell r="P21">
-            <v>2.6725462684572727E-2</v>
-          </cell>
-        </row>
-        <row r="22">
-          <cell r="B22">
-            <v>2</v>
-          </cell>
-          <cell r="C22" t="str">
-            <v xml:space="preserve"> Trasporto materie prime a reparto</v>
-          </cell>
-          <cell r="F22">
-            <v>2</v>
-          </cell>
-          <cell r="G22">
-            <v>8</v>
-          </cell>
-          <cell r="H22">
-            <v>8</v>
-          </cell>
-          <cell r="I22">
-            <v>16</v>
-          </cell>
-          <cell r="K22">
-            <v>59868</v>
-          </cell>
-          <cell r="L22">
-            <v>2.6725462684572727E-2</v>
-          </cell>
-          <cell r="M22">
-            <v>2.6725462684572727E-2</v>
-          </cell>
-          <cell r="N22">
-            <v>2.6725462684572727E-2</v>
-          </cell>
-          <cell r="O22">
-            <v>2.6725462684572727E-2</v>
-          </cell>
-          <cell r="P22">
-            <v>2.6725462684572727E-2</v>
-          </cell>
-        </row>
-        <row r="23">
-          <cell r="B23">
-            <v>3</v>
-          </cell>
-          <cell r="C23" t="str">
-            <v xml:space="preserve"> Lavaggio palbox m.p. + travaso da cartonbox altri</v>
-          </cell>
-          <cell r="F23">
-            <v>2</v>
-          </cell>
-          <cell r="G23">
-            <v>8</v>
-          </cell>
-          <cell r="H23">
-            <v>8</v>
-          </cell>
-          <cell r="I23">
-            <v>16</v>
-          </cell>
-          <cell r="K23">
-            <v>59868</v>
-          </cell>
-          <cell r="L23">
-            <v>2.6725462684572727E-2</v>
-          </cell>
-          <cell r="M23">
-            <v>2.6725462684572727E-2</v>
-          </cell>
-          <cell r="N23">
-            <v>2.6725462684572727E-2</v>
-          </cell>
-          <cell r="O23">
-            <v>2.6725462684572727E-2</v>
-          </cell>
-          <cell r="P23">
-            <v>2.6725462684572727E-2</v>
-          </cell>
-        </row>
-        <row r="24">
-          <cell r="C24" t="str">
-            <v xml:space="preserve"> Analisi materie prime</v>
-          </cell>
-          <cell r="G24">
-            <v>8</v>
-          </cell>
-          <cell r="H24">
-            <v>0</v>
-          </cell>
-          <cell r="I24">
-            <v>0</v>
-          </cell>
-          <cell r="K24">
-            <v>22660</v>
-          </cell>
-          <cell r="L24">
-            <v>0</v>
-          </cell>
-          <cell r="M24">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="25">
-          <cell r="B25" t="str">
-            <v>B</v>
-          </cell>
-        </row>
-        <row r="26">
-          <cell r="C26" t="str">
-            <v xml:space="preserve"> PREPARAZIONI IMPASTI E FUSIONE</v>
-          </cell>
-        </row>
-        <row r="27">
-          <cell r="B27">
-            <v>1</v>
-          </cell>
-          <cell r="C27" t="str">
-            <v xml:space="preserve"> Impostazione ricette + carico + analisi</v>
-          </cell>
-          <cell r="F27">
-            <v>2</v>
-          </cell>
-          <cell r="G27">
-            <v>8</v>
-          </cell>
-          <cell r="H27">
-            <v>8</v>
-          </cell>
-          <cell r="I27">
-            <v>16</v>
-          </cell>
-          <cell r="K27">
-            <v>22660</v>
-          </cell>
-          <cell r="L27">
-            <v>7.0609002647837593E-2</v>
-          </cell>
-          <cell r="M27">
-            <v>7.0609002647837593E-2</v>
-          </cell>
-        </row>
-        <row r="29">
-          <cell r="B29">
-            <v>2</v>
-          </cell>
-          <cell r="C29" t="str">
-            <v xml:space="preserve"> Assistenza impianto sterilizzazione e cremificazione</v>
-          </cell>
-          <cell r="F29">
-            <v>2</v>
-          </cell>
-          <cell r="G29">
-            <v>8</v>
-          </cell>
-          <cell r="H29">
-            <v>8</v>
-          </cell>
-          <cell r="I29">
-            <v>16</v>
-          </cell>
-          <cell r="K29">
-            <v>22660</v>
-          </cell>
-          <cell r="L29">
-            <v>7.0609002647837593E-2</v>
-          </cell>
-          <cell r="M29">
-            <v>7.0609002647837593E-2</v>
-          </cell>
-        </row>
-        <row r="30">
-          <cell r="C30" t="str">
-            <v xml:space="preserve"> Stephan + preparazione e carico caseina</v>
-          </cell>
-        </row>
-        <row r="31">
-          <cell r="B31">
-            <v>3</v>
-          </cell>
-          <cell r="C31" t="str">
-            <v xml:space="preserve"> Carico burro, fusione burro </v>
-          </cell>
-          <cell r="G31">
-            <v>0</v>
-          </cell>
-          <cell r="H31">
-            <v>0</v>
-          </cell>
-          <cell r="I31">
-            <v>0</v>
-          </cell>
-          <cell r="K31">
-            <v>22660</v>
-          </cell>
-          <cell r="L31">
-            <v>0</v>
-          </cell>
-          <cell r="M31">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="33">
-          <cell r="B33">
-            <v>4</v>
-          </cell>
-          <cell r="C33" t="str">
-            <v xml:space="preserve"> Assistenza e controllo cremificazione</v>
-          </cell>
-          <cell r="H33">
-            <v>0</v>
-          </cell>
-          <cell r="I33">
-            <v>0</v>
-          </cell>
-          <cell r="K33">
-            <v>22660</v>
-          </cell>
-          <cell r="L33">
-            <v>0</v>
-          </cell>
-          <cell r="M33">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="34">
-          <cell r="B34">
-            <v>5</v>
-          </cell>
-          <cell r="C34" t="str">
-            <v xml:space="preserve"> Cottura in 1 Ks : addetti Stephan + pesatura sali di fusione</v>
-          </cell>
-          <cell r="H34">
-            <v>0</v>
-          </cell>
-          <cell r="I34">
-            <v>0</v>
-          </cell>
-          <cell r="K34">
-            <v>22660</v>
-          </cell>
-          <cell r="L34">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="35">
-          <cell r="B35">
-            <v>6</v>
-          </cell>
-          <cell r="C35" t="str">
-            <v xml:space="preserve"> Pressatura porzioni fusi + filante</v>
-          </cell>
-          <cell r="H35">
-            <v>0</v>
-          </cell>
-          <cell r="I35">
-            <v>0</v>
-          </cell>
-          <cell r="K35">
-            <v>59868</v>
-          </cell>
-          <cell r="L35">
-            <v>0</v>
-          </cell>
-          <cell r="M35">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="37">
-          <cell r="B37">
-            <v>7</v>
-          </cell>
-          <cell r="C37" t="str">
-            <v xml:space="preserve"> Preparazione e cottura form. prefuso settimanale</v>
-          </cell>
-          <cell r="H37">
-            <v>0</v>
-          </cell>
-          <cell r="I37">
-            <v>0</v>
-          </cell>
-          <cell r="K37">
-            <v>113300</v>
-          </cell>
-          <cell r="L37">
-            <v>0</v>
-          </cell>
-          <cell r="M37">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="39">
-          <cell r="B39">
-            <v>8</v>
-          </cell>
-          <cell r="C39" t="str">
-            <v xml:space="preserve"> Colatura linee + trasporto pasta a Stephan</v>
-          </cell>
-          <cell r="F39">
-            <v>2</v>
-          </cell>
-          <cell r="G39">
-            <v>8</v>
-          </cell>
-          <cell r="H39">
-            <v>8</v>
-          </cell>
-          <cell r="I39">
-            <v>16</v>
-          </cell>
-          <cell r="K39">
-            <v>29528</v>
-          </cell>
-          <cell r="L39">
-            <v>5.4185857491194797E-2</v>
-          </cell>
-          <cell r="M39">
-            <v>5.4185857491194797E-2</v>
-          </cell>
-        </row>
-        <row r="41">
-          <cell r="B41">
-            <v>9</v>
-          </cell>
-          <cell r="C41" t="str">
-            <v xml:space="preserve"> Lavaggio iniziale e finale Stephan</v>
-          </cell>
-          <cell r="F41">
-            <v>1</v>
-          </cell>
-          <cell r="G41">
-            <v>8</v>
-          </cell>
-          <cell r="H41">
-            <v>8</v>
-          </cell>
-          <cell r="I41">
-            <v>8</v>
-          </cell>
-          <cell r="K41">
-            <v>22660</v>
-          </cell>
-          <cell r="L41">
-            <v>3.5304501323918797E-2</v>
-          </cell>
-          <cell r="M41">
-            <v>3.5304501323918797E-2</v>
-          </cell>
-        </row>
-        <row r="43">
-          <cell r="B43">
-            <v>10</v>
-          </cell>
-          <cell r="C43" t="str">
-            <v xml:space="preserve"> Lavaggio iniziale + finale Combinator e linee, preparazione</v>
-          </cell>
-          <cell r="G43">
-            <v>8</v>
-          </cell>
-          <cell r="H43">
-            <v>8</v>
-          </cell>
-          <cell r="I43">
-            <v>0</v>
-          </cell>
-          <cell r="K43">
-            <v>29528</v>
-          </cell>
-          <cell r="L43">
-            <v>0</v>
-          </cell>
-          <cell r="M43">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="44">
-          <cell r="C44" t="str">
-            <v xml:space="preserve"> macchine formatrici e lavaggio allibert</v>
-          </cell>
-        </row>
-        <row r="46">
-          <cell r="B46">
-            <v>11</v>
-          </cell>
-          <cell r="C46" t="str">
-            <v>Lavaggio ferri</v>
-          </cell>
-          <cell r="F46">
-            <v>1</v>
-          </cell>
-          <cell r="G46">
-            <v>8</v>
-          </cell>
-          <cell r="H46">
-            <v>8</v>
-          </cell>
-          <cell r="I46">
-            <v>8</v>
-          </cell>
-          <cell r="K46">
-            <v>29528</v>
-          </cell>
-          <cell r="L46">
-            <v>2.7092928745597399E-2</v>
-          </cell>
-          <cell r="M46">
-            <v>2.7092928745597399E-2</v>
-          </cell>
-        </row>
-        <row r="48">
-          <cell r="B48">
-            <v>12</v>
-          </cell>
-          <cell r="C48" t="str">
-            <v>Travaso pasta a fusione da cartonbox a palbox</v>
-          </cell>
-          <cell r="H48">
-            <v>0</v>
-          </cell>
-          <cell r="I48">
-            <v>0</v>
-          </cell>
-          <cell r="K48">
-            <v>29528</v>
-          </cell>
-          <cell r="L48">
-            <v>0</v>
-          </cell>
-          <cell r="M48">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="49">
-          <cell r="C49" t="str">
-            <v xml:space="preserve"> Addetti Ks x Dolc. Cr. / CBP +/ 4 Form. / Process./ Tiramisù</v>
-          </cell>
-          <cell r="F49">
-            <v>2</v>
-          </cell>
-          <cell r="G49">
-            <v>8</v>
-          </cell>
-          <cell r="H49">
-            <v>8</v>
-          </cell>
-          <cell r="I49">
-            <v>16</v>
-          </cell>
-          <cell r="K49">
-            <v>6868</v>
-          </cell>
-          <cell r="L49">
-            <v>0.23296447291788003</v>
-          </cell>
-          <cell r="N49">
-            <v>0.23296447291788003</v>
-          </cell>
-        </row>
-        <row r="50">
-          <cell r="C50" t="str">
-            <v xml:space="preserve"> Capi reparto (vedi scheda allegato 3)</v>
-          </cell>
-          <cell r="L50">
-            <v>1.2026458208057728E-2</v>
-          </cell>
-          <cell r="M50">
-            <v>1.2026458208057728E-2</v>
-          </cell>
-          <cell r="N50">
-            <v>1.2026458208057728E-2</v>
-          </cell>
-          <cell r="O50">
-            <v>1.2026458208057728E-2</v>
-          </cell>
-          <cell r="P50">
-            <v>1.2026458208057728E-2</v>
-          </cell>
-        </row>
-        <row r="52">
-          <cell r="C52" t="str">
-            <v>NB  tener conto di 1 x 8 ore Magor</v>
-          </cell>
-          <cell r="F52">
-            <v>1</v>
-          </cell>
-          <cell r="G52">
-            <v>8</v>
-          </cell>
-          <cell r="H52">
-            <v>8</v>
-          </cell>
-          <cell r="I52">
-            <v>8</v>
-          </cell>
-        </row>
-        <row r="56">
-          <cell r="C56" t="str">
-            <v xml:space="preserve"> TEMPO TOTALE</v>
-          </cell>
-          <cell r="E56" t="str">
-            <v>ORE/100 KG.</v>
-          </cell>
-          <cell r="I56">
-            <v>136</v>
-          </cell>
-          <cell r="L56">
-            <v>0.58296861203604211</v>
-          </cell>
-          <cell r="M56">
-            <v>0.35000413911816208</v>
-          </cell>
-          <cell r="N56">
-            <v>0.32516731917965591</v>
-          </cell>
-          <cell r="O56">
-            <v>9.2202846261775911E-2</v>
-          </cell>
-          <cell r="P56">
-            <v>9.2202846261775911E-2</v>
-          </cell>
-        </row>
-        <row r="60">
-          <cell r="C60" t="str">
-            <v xml:space="preserve"> Determinanti 2004</v>
-          </cell>
-          <cell r="F60" t="str">
-            <v>KG/ANNO</v>
-          </cell>
-          <cell r="G60" t="str">
-            <v>GG/ANNO</v>
-          </cell>
-          <cell r="H60" t="str">
-            <v>KG/GIORNO</v>
-          </cell>
-        </row>
-        <row r="61">
-          <cell r="C61" t="str">
-            <v xml:space="preserve"> C.B.P. Normale</v>
-          </cell>
-          <cell r="F61">
-            <v>5665000</v>
-          </cell>
-          <cell r="G61">
-            <v>250</v>
-          </cell>
-          <cell r="H61">
-            <v>22660</v>
-          </cell>
-          <cell r="K61" t="str">
-            <v xml:space="preserve"> SEGUE SU SCHEDE DI CONFEZIONAMENTO</v>
-          </cell>
-        </row>
-        <row r="62">
-          <cell r="C62" t="str">
-            <v xml:space="preserve"> C.B.P. +,  Dolcelatte cremoso, Crema 4 formaggi, Processato</v>
-          </cell>
-          <cell r="F62">
-            <v>1717000</v>
-          </cell>
-          <cell r="G62">
-            <v>250</v>
-          </cell>
-          <cell r="H62">
-            <v>6868</v>
-          </cell>
-          <cell r="K62" t="str">
-            <v xml:space="preserve"> - FUSI PORZIONI</v>
-          </cell>
-        </row>
-        <row r="63">
-          <cell r="H63" t="str">
-            <v/>
-          </cell>
-          <cell r="K63" t="str">
-            <v xml:space="preserve"> - FILANTE</v>
-          </cell>
-        </row>
-        <row r="64">
-          <cell r="C64" t="str">
-            <v xml:space="preserve"> Filante + Idea Pizza + Fil. Rapè + Filone Mozz.</v>
-          </cell>
-          <cell r="F64">
-            <v>7585000</v>
-          </cell>
-          <cell r="G64">
-            <v>250</v>
-          </cell>
-          <cell r="H64">
-            <v>30340</v>
-          </cell>
-          <cell r="K64" t="str">
-            <v xml:space="preserve"> - FILANTE x PIZZA</v>
-          </cell>
-        </row>
-        <row r="65">
-          <cell r="K65" t="str">
-            <v xml:space="preserve"> - IDEA PIZZA</v>
-          </cell>
-        </row>
-        <row r="66">
-          <cell r="K66" t="str">
-            <v xml:space="preserve"> - FORMAGGIO PER PIZZA</v>
-          </cell>
-        </row>
-        <row r="68">
-          <cell r="C68" t="str">
-            <v xml:space="preserve"> TOTALI</v>
-          </cell>
-          <cell r="F68">
-            <v>14967000</v>
-          </cell>
-          <cell r="G68">
-            <v>248</v>
-          </cell>
-          <cell r="H68">
-            <v>59868</v>
-          </cell>
-        </row>
-      </sheetData>
+      <sheetData sheetId="0" refreshError="1"/>
       <sheetData sheetId="1"/>
       <sheetData sheetId="2"/>
       <sheetData sheetId="3"/>
@@ -2813,13 +1430,7 @@
     </sheetNames>
     <sheetDataSet>
       <sheetData sheetId="0"/>
-      <sheetData sheetId="1" refreshError="1">
-        <row r="3">
-          <cell r="A3" t="str">
-            <v>_Amount_for_Monthly</v>
-          </cell>
-        </row>
-      </sheetData>
+      <sheetData sheetId="1" refreshError="1"/>
       <sheetData sheetId="2"/>
       <sheetData sheetId="3"/>
       <sheetData sheetId="4"/>
@@ -2881,18 +1492,7 @@
       <sheetData sheetId="7" refreshError="1"/>
       <sheetData sheetId="8" refreshError="1"/>
       <sheetData sheetId="9" refreshError="1"/>
-      <sheetData sheetId="10">
-        <row r="2">
-          <cell r="AR2">
-            <v>0.83</v>
-          </cell>
-        </row>
-        <row r="3">
-          <cell r="AR3">
-            <v>1.27</v>
-          </cell>
-        </row>
-      </sheetData>
+      <sheetData sheetId="10"/>
       <sheetData sheetId="11" refreshError="1"/>
       <sheetData sheetId="12" refreshError="1"/>
       <sheetData sheetId="13" refreshError="1"/>
@@ -2903,13 +1503,7 @@
       <sheetData sheetId="18" refreshError="1"/>
       <sheetData sheetId="19" refreshError="1"/>
       <sheetData sheetId="20" refreshError="1"/>
-      <sheetData sheetId="21">
-        <row r="6">
-          <cell r="H6">
-            <v>82589</v>
-          </cell>
-        </row>
-      </sheetData>
+      <sheetData sheetId="21"/>
       <sheetData sheetId="22"/>
       <sheetData sheetId="23" refreshError="1"/>
       <sheetData sheetId="24" refreshError="1"/>
@@ -2980,117 +1574,16 @@
     <sheetDataSet>
       <sheetData sheetId="0"/>
       <sheetData sheetId="1"/>
-      <sheetData sheetId="2" refreshError="1">
-        <row r="3">
-          <cell r="B3">
-            <v>1</v>
-          </cell>
-          <cell r="C3" t="str">
-            <v>JANVIER</v>
-          </cell>
-        </row>
-        <row r="4">
-          <cell r="B4">
-            <v>2</v>
-          </cell>
-          <cell r="C4" t="str">
-            <v>FÉVRIER</v>
-          </cell>
-        </row>
-        <row r="5">
-          <cell r="B5">
-            <v>3</v>
-          </cell>
-          <cell r="C5" t="str">
-            <v>MARS</v>
-          </cell>
-        </row>
-        <row r="6">
-          <cell r="B6">
-            <v>4</v>
-          </cell>
-          <cell r="C6" t="str">
-            <v>AVRIL</v>
-          </cell>
-        </row>
-        <row r="7">
-          <cell r="B7">
-            <v>5</v>
-          </cell>
-          <cell r="C7" t="str">
-            <v>MAI</v>
-          </cell>
-        </row>
-        <row r="8">
-          <cell r="B8">
-            <v>6</v>
-          </cell>
-          <cell r="C8" t="str">
-            <v>JUIN</v>
-          </cell>
-        </row>
-        <row r="9">
-          <cell r="B9">
-            <v>7</v>
-          </cell>
-          <cell r="C9" t="str">
-            <v>JUILLET</v>
-          </cell>
-        </row>
-        <row r="10">
-          <cell r="B10">
-            <v>8</v>
-          </cell>
-          <cell r="C10" t="str">
-            <v>AOÛT</v>
-          </cell>
-        </row>
-        <row r="11">
-          <cell r="B11">
-            <v>9</v>
-          </cell>
-          <cell r="C11" t="str">
-            <v>SEPTEMBRE</v>
-          </cell>
-        </row>
-        <row r="12">
-          <cell r="B12">
-            <v>10</v>
-          </cell>
-          <cell r="C12" t="str">
-            <v>OCTOBRE</v>
-          </cell>
-        </row>
-        <row r="13">
-          <cell r="B13">
-            <v>11</v>
-          </cell>
-          <cell r="C13" t="str">
-            <v>NOVEMBRE</v>
-          </cell>
-        </row>
-        <row r="14">
-          <cell r="B14">
-            <v>12</v>
-          </cell>
-          <cell r="C14" t="str">
-            <v>DÉCEMBRE</v>
-          </cell>
-        </row>
-      </sheetData>
+      <sheetData sheetId="2" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -3128,7 +1621,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -3234,7 +1727,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -3376,7 +1869,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -3388,36 +1881,36 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G22"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="48.7109375" customWidth="1"/>
     <col min="2" max="2" width="14.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="21" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="21">
       <c r="A1" s="5" t="s">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="B1" s="15" t="s">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="C1" s="15" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D1" s="15" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="15" t="s">
+      <c r="G1" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="15" t="s">
-        <v>38</v>
-      </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7">
       <c r="A2" s="17" t="s">
         <v>7</v>
       </c>
@@ -3438,9 +1931,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" ht="18.75">
       <c r="A3" s="22" t="s">
-        <v>34</v>
+        <v>8</v>
       </c>
       <c r="B3" s="23"/>
       <c r="C3" s="23"/>
@@ -3449,9 +1942,9 @@
       <c r="F3" s="23"/>
       <c r="G3" s="23"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7">
       <c r="A4" s="20" t="s">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2">
@@ -3470,9 +1963,9 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7">
       <c r="A5" s="21" t="s">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3">
@@ -3491,12 +1984,12 @@
         <v>0.18</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7">
       <c r="A6" s="1" t="s">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="B6" s="36" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="C6" s="6">
         <f>C4-C5</f>
@@ -3519,12 +2012,12 @@
         <v>0.22000000000000003</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7">
       <c r="A7" s="1" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="B7" s="37" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="C7" s="7">
         <f>(1-C4)/(1-C5)</f>
@@ -3547,12 +2040,12 @@
         <v>0.7317073170731706</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7">
       <c r="A8" s="4" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="B8" s="38" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="C8" s="8">
         <f>C5/C4</f>
@@ -3575,9 +2068,9 @@
         <v>0.44999999999999996</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" ht="18.75">
       <c r="A9" s="24" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
       <c r="B9" s="25"/>
       <c r="C9" s="25"/>
@@ -3586,9 +2079,9 @@
       <c r="F9" s="25"/>
       <c r="G9" s="25"/>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7">
       <c r="A10" s="26" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B10" s="27"/>
       <c r="C10" s="27">
@@ -3607,9 +2100,9 @@
         <v>38.1</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7">
       <c r="A11" s="28" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B11" s="29"/>
       <c r="C11" s="29">
@@ -3628,9 +2121,9 @@
         <v>32.1</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" ht="18.75">
       <c r="A12" s="30" t="s">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="B12" s="31"/>
       <c r="C12" s="31"/>
@@ -3639,9 +2132,9 @@
       <c r="F12" s="31"/>
       <c r="G12" s="31"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7">
       <c r="A13" s="32" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="B13" s="33"/>
       <c r="C13" s="33">
@@ -3660,9 +2153,9 @@
         <v>0.9446</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" ht="18.75">
       <c r="A14" s="19" t="s">
-        <v>37</v>
+        <v>22</v>
       </c>
       <c r="B14" s="34"/>
       <c r="C14" s="34"/>
@@ -3671,12 +2164,12 @@
       <c r="F14" s="34"/>
       <c r="G14" s="34"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7">
       <c r="A15" s="1" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="B15" s="39" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C15" s="9">
         <f>C13*C11</f>
@@ -3699,12 +2192,12 @@
         <v>30.321660000000001</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7">
       <c r="A16" s="1" t="s">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="B16" s="40" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C16" s="16">
         <f>C6*1000/C15</f>
@@ -3727,12 +2220,12 @@
         <v>7.2555394394634076</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7">
       <c r="A17" s="1" t="s">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="B17" s="39" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C17" s="9">
         <f>C5*1000/C16</f>
@@ -3755,12 +2248,12 @@
         <v>24.808630909090905</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7">
       <c r="A18" s="1" t="s">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="B18" s="41" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="C18" s="14">
         <f>C17/C10</f>
@@ -3783,12 +2276,12 @@
         <v>0.65114516821760904</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7">
       <c r="A19" s="12" t="s">
-        <v>16</v>
+        <v>31</v>
       </c>
       <c r="B19" s="42" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C19" s="13">
         <f>C17-C10</f>
@@ -3811,12 +2304,12 @@
         <v>-13.291369090909097</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7">
       <c r="A20" s="4" t="s">
-        <v>12</v>
+        <v>33</v>
       </c>
       <c r="B20" s="43" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="C20" s="35">
         <f>C19/C10</f>
@@ -3839,12 +2332,12 @@
         <v>-0.34885483178239096</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7">
       <c r="A21" s="12" t="s">
-        <v>13</v>
+        <v>35</v>
       </c>
       <c r="B21" s="44" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="C21" s="10">
         <f>C10*C16</f>
@@ -3867,12 +2360,12 @@
         <v>276.43605264355585</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7">
       <c r="A22" s="4" t="s">
-        <v>11</v>
+        <v>37</v>
       </c>
       <c r="B22" s="45" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="C22" s="11">
         <f>C11*C16</f>

</xml_diff>